<commit_message>
updated and exported supplementary tables for the manuscript
</commit_message>
<xml_diff>
--- a/data/TableS2_point_intercept_summary.xlsx
+++ b/data/TableS2_point_intercept_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
   <si>
     <t xml:space="preserve">species</t>
   </si>
@@ -253,6 +253,12 @@
   </si>
   <si>
     <t xml:space="preserve">Vaccinium vitis-idaea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proportion damaged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total nr intercepts</t>
   </si>
 </sst>
 </file>
@@ -5349,6 +5355,196 @@
         <v>0</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>80</v>
+      </c>
+      <c r="B51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T51" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="U51" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="V51" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="W51" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="X51" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>81</v>
+      </c>
+      <c r="B52" t="n">
+        <v>200</v>
+      </c>
+      <c r="C52" t="n">
+        <v>200</v>
+      </c>
+      <c r="D52" t="n">
+        <v>200</v>
+      </c>
+      <c r="E52" t="n">
+        <v>200</v>
+      </c>
+      <c r="F52" t="n">
+        <v>200</v>
+      </c>
+      <c r="G52" t="n">
+        <v>200</v>
+      </c>
+      <c r="H52" t="n">
+        <v>200</v>
+      </c>
+      <c r="I52" t="n">
+        <v>200</v>
+      </c>
+      <c r="J52" t="n">
+        <v>200</v>
+      </c>
+      <c r="K52" t="n">
+        <v>200</v>
+      </c>
+      <c r="L52" t="n">
+        <v>100</v>
+      </c>
+      <c r="M52" t="n">
+        <v>100</v>
+      </c>
+      <c r="N52" t="n">
+        <v>200</v>
+      </c>
+      <c r="O52" t="n">
+        <v>200</v>
+      </c>
+      <c r="P52" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>200</v>
+      </c>
+      <c r="R52" t="n">
+        <v>200</v>
+      </c>
+      <c r="S52" t="n">
+        <v>100</v>
+      </c>
+      <c r="T52" t="n">
+        <v>200</v>
+      </c>
+      <c r="U52" t="n">
+        <v>200</v>
+      </c>
+      <c r="V52" t="n">
+        <v>200</v>
+      </c>
+      <c r="W52" t="n">
+        <v>200</v>
+      </c>
+      <c r="X52" t="n">
+        <v>200</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>200</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>200</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>200</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>200</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>